<commit_message>
Add Site Ops Page Names suite and CWV PoP sort/export coverage.
Introduce BI Site Operations Dashboard for Page Names regression (POM, probe, Excel) and extend CWV Top 10 PoP with column-sort and Export chart hamburger soft checks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/CWV_Top10_Period_over_Period_PoP_Regression.xlsx
+++ b/docs/CWV_Top10_Period_over_Period_PoP_Regression.xlsx
@@ -13,9 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="151">
-  <si>
-    <t>Profile: US / GDC Test Site 2 | Type: Regression (reversible Lookback/filter + disposable Save As) | Total TCs: 23 | CWV Top 10 Period over Period (PoP)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="161">
+  <si>
+    <t>Profile: US / GDC Test Site 2 | Type: Regression (reversible Lookback/filter/sort + disposable Save As + soft export) | Total TCs: 25 | CWV Top 10 Period over Period (PoP)</t>
   </si>
   <si>
     <t>SoT = PDF BI Dashboard CWV Top 10 PoP + live #bi-iframe probe. Suite home: Business Intelligence → Dashboards → CWV Top 10 Period over Period (PoP).</t>
@@ -138,13 +138,25 @@
     <t>REG-CWV-POP-022</t>
   </si>
   <si>
+    <t>Sort</t>
+  </si>
+  <si>
+    <t>REG-CWV-POP-024</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>REG-CWV-POP-025</t>
+  </si>
+  <si>
     <t>TOTAL</t>
   </si>
   <si>
     <t>REG-CWV-POP-001 .. REG-CWV-POP-023</t>
   </si>
   <si>
-    <t>Execution: Passed (23/23 + auth setup) — Executed 2026-08-26 on GDC Test Site 2 (US). Allure: allure_reports/cwv-pop-report/index.html. Soft annotations: Google CWV band labels soft-miss in body sample (Delta Definitions present); Comparison Method/Period host soft-miss (live Lookback uses Last N Complete Month + Day/Week); Lookback Apply signature often unchanged; Refresh Data signature identical OK; leftover Save As clone CWV-PoP-QA-mta03xct needs manual cleanup if still listed; portal site Select2 may soft-hide on BI shell.</t>
+    <t>Execution: Passed (25/25 + auth; sort+export added) — Executed 2026-08-27 after adding REG-CWV-POP-024 (column sort) and REG-CWV-POP-025 (Export PNG/PDF/PPT). Soft: sort 6/6 headers clicked, order identical; Export PDF download Onload_*.pdf; PNG/PPT soft-miss; leftover clone CWV-PoP-QA-mtb874hp. Allure: allure_reports/cwv-pop-report/index.html</t>
   </si>
   <si>
     <t>Test Case ID</t>
@@ -180,7 +192,7 @@
 3. #bi-iframe attached.</t>
   </si>
   <si>
-    <t>Passed (23/23 + auth setup)</t>
+    <t>Passed (25/25 + auth; sort+export added)</t>
   </si>
   <si>
     <t>GDC Test Site 2; iframe ready; PoP identity</t>
@@ -415,15 +427,15 @@
     <t>1. Only CWV Top 10 PoP in BI tool.</t>
   </si>
   <si>
-    <t>Lookback → filter → Refresh → Reset soft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Chain mutations
+    <t>Lookback → filter → sort → Refresh → Reset soft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Chain Lookback, Device filter, Page Name sort, Refresh
 2. Reset.</t>
   </si>
   <si>
     <t xml:space="preserve">1. PoP identity retained
-2. filters restored soft.</t>
+2. filters/sort restored soft.</t>
   </si>
   <si>
     <t>REG-CWV-POP-021</t>
@@ -451,6 +463,32 @@
 2. PoP soft.</t>
   </si>
   <si>
+    <t>Column sort all visible grid headers; rows rearrange soft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click each sortable header on Page Name tables
+2. assert row order soft
+3. Reset.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Headers clickable
+2. order changes or annotate equal values.</t>
+  </si>
+  <si>
+    <t>Export chart hamburger PNG/PDF/PowerPoint soft vs UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Export chart
+2. assert PNG/PDF/PPT (or CSV)
+3. soft export
+4. cross-check UI labels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Menu options soft
+2. downloads soft
+3. PoP identity + LCP/Page Name retained.</t>
+  </si>
+  <si>
     <t>REG-CWV-POP-023</t>
   </si>
   <si>
@@ -472,7 +510,7 @@
     <t>Profile / Site: US — GDC Test Site 2</t>
   </si>
   <si>
-    <t>Type: Regression (reversible Lookback/filter + disposable Save As). Prefer live UI; do not assert exact backend numeric values unless specified.</t>
+    <t>Type: Regression (reversible Lookback/filter/sort + disposable Save As + soft export). Prefer live UI; do not assert exact backend numeric values unless specified.</t>
   </si>
   <si>
     <t>Columns: Test Case ID | Type | Module | Submodule | Title | Steps | Expected Results | Status</t>
@@ -481,16 +519,16 @@
     <t>Header style: bold white text on #1F4E79</t>
   </si>
   <si>
-    <t>Total cases: 23 (REG-CWV-POP-001 .. REG-CWV-POP-023)</t>
+    <t>Total cases: 25 (REG-CWV-POP-001 .. REG-CWV-POP-023)</t>
   </si>
   <si>
     <t>Automation: tests/regression_tests/US2/advanced-reporting/custom-reporting/business-intelligence/cwv-top10-pop/cwv.top10.pop.regression.spec.ts</t>
   </si>
   <si>
-    <t>Execution status: Passed (23/23 + auth setup)</t>
-  </si>
-  <si>
-    <t>Execution note: Executed 2026-08-26 on GDC Test Site 2 (US). Allure: allure_reports/cwv-pop-report/index.html. Soft annotations: Google CWV band labels soft-miss in body sample (Delta Definitions present); Comparison Method/Period host soft-miss (live Lookback uses Last N Complete Month + Day/Week); Lookback Apply signature often unchanged; Refresh Data signature identical OK; leftover Save As clone CWV-PoP-QA-mta03xct needs manual cleanup if still listed; portal site Select2 may soft-hide on BI shell.</t>
+    <t>Execution status: Passed (25/25 + auth; sort+export added)</t>
+  </si>
+  <si>
+    <t>Execution note: Executed 2026-08-27 after adding REG-CWV-POP-024 (column sort) and REG-CWV-POP-025 (Export PNG/PDF/PPT). Soft: sort 6/6 headers clicked, order identical; Export PDF download Onload_*.pdf; PNG/PPT soft-miss; leftover clone CWV-PoP-QA-mtb874hp. Allure: allure_reports/cwv-pop-report/index.html</t>
   </si>
   <si>
     <t>Exact home: Advanced Reporting &amp; Alerting / Custom Reporting / Business Intelligence / Dashboards / CWV Top 10 Period over Period (PoP).</t>
@@ -499,7 +537,7 @@
     <t>Never accept VitalPulse, VitalScope (Core Web Vitals), Native App Top 10 PoP, or portal site/dashboard as suite home.</t>
   </si>
   <si>
-    <t>All widgets/filters live inside #bi-iframe (jbi.bluetriangletech.com). Do not assert portal body alone.</t>
+    <t>All widgets/filters/sort/export live inside #bi-iframe (jbi.bluetriangletech.com). Do not assert portal body alone.</t>
   </si>
   <si>
     <t>Portal #toggle-filters is NOT BI Lookback Period.</t>
@@ -511,7 +549,7 @@
     <t>Catalog ~13 widgets soft; prefer PDF five + tables as primary inventory.</t>
   </si>
   <si>
-    <t>Lookback ± months + Apply; filter combos; Save As clone; Refresh Data; Reset to Default — restore all mutations.</t>
+    <t>Lookback ± months + Apply; filter combos; column sort all headers; Export chart PNG/PDF/PPT soft; Save As clone; Refresh Data; Reset to Default — restore all mutations.</t>
   </si>
   <si>
     <t>Do not create permanent Schedules / AI Query assets / overwrite Global PoP.</t>
@@ -932,7 +970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1209,33 +1247,61 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="6" t="s">
+    <row r="21" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="5">
+        <v>1</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="5">
+        <v>1</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="6">
-        <v>23</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="D23" s="6">
+        <v>25</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1244,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1259,10 +1325,10 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
@@ -1271,16 +1337,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1288,7 +1354,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>8</v>
@@ -1297,16 +1363,16 @@
         <v>19</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1314,7 +1380,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>8</v>
@@ -1323,16 +1389,16 @@
         <v>21</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1340,7 +1406,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>8</v>
@@ -1349,24 +1415,24 @@
         <v>23</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>8</v>
@@ -1375,24 +1441,24 @@
         <v>13</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>8</v>
@@ -1401,16 +1467,16 @@
         <v>13</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1418,7 +1484,7 @@
         <v>26</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>8</v>
@@ -1427,16 +1493,16 @@
         <v>25</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1444,7 +1510,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>8</v>
@@ -1453,16 +1519,16 @@
         <v>27</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1470,7 +1536,7 @@
         <v>30</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>8</v>
@@ -1479,16 +1545,16 @@
         <v>29</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1496,7 +1562,7 @@
         <v>32</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>8</v>
@@ -1505,24 +1571,24 @@
         <v>31</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>8</v>
@@ -1531,24 +1597,24 @@
         <v>15</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>8</v>
@@ -1557,24 +1623,24 @@
         <v>15</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>8</v>
@@ -1583,24 +1649,24 @@
         <v>9</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>8</v>
@@ -1609,24 +1675,24 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>8</v>
@@ -1635,24 +1701,24 @@
         <v>9</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>8</v>
@@ -1661,24 +1727,24 @@
         <v>11</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>8</v>
@@ -1687,24 +1753,24 @@
         <v>11</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>8</v>
@@ -1713,16 +1779,16 @@
         <v>11</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1730,7 +1796,7 @@
         <v>34</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>8</v>
@@ -1739,16 +1805,16 @@
         <v>33</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1756,7 +1822,7 @@
         <v>36</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>8</v>
@@ -1765,16 +1831,16 @@
         <v>35</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1782,7 +1848,7 @@
         <v>38</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>8</v>
@@ -1791,24 +1857,24 @@
         <v>37</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>8</v>
@@ -1817,16 +1883,16 @@
         <v>17</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1834,7 +1900,7 @@
         <v>40</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>8</v>
@@ -1843,50 +1909,102 @@
         <v>39</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>129</v>
+        <v>42</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E24" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>54</v>
+      <c r="E26" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H10:H24">
+    <dataValidation type="list" allowBlank="1" sqref="H10:H26">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H24">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H26">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1905,37 +2023,37 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -1945,57 +2063,57 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>